<commit_message>
chore: run 2026-03-24 12:40 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_24_03_2026.xlsx
+++ b/logs/Consolidado_24_03_2026.xlsx
@@ -638,10 +638,10 @@
         <v>151</v>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -657,10 +657,10 @@
         <v>66</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -676,10 +676,10 @@
         <v>80</v>
       </c>
       <c r="C4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -695,10 +695,10 @@
         <v>70</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>2</v>
@@ -714,10 +714,10 @@
         <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -1148,40 +1148,40 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Body Gentle Scrub for Sensitive Skin
 Esfoliante de Corpo Suave Pele Sensível
 200 ml</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/body-gentle-scrub-for-sensitive-skin-6545160.html</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>6545160</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -4369,40 +4369,40 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B90" s="7" t="inlineStr">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C90" s="7" t="inlineStr">
+      <c r="C90" s="5" t="inlineStr">
         <is>
           <t>Milk Cleanser Dry Sensitive Skin
 Leite de Limpeza Desmaquilhante Pele Seca
 200 ml</t>
         </is>
       </c>
-      <c r="D90" s="7" t="inlineStr">
+      <c r="D90" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/milk-cleanser-dry-sensitive-skin-3001085.html</t>
         </is>
       </c>
-      <c r="E90" s="7" t="inlineStr"/>
-      <c r="F90" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G90" s="7" t="inlineStr">
+      <c r="E90" s="5" t="inlineStr"/>
+      <c r="F90" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
         <is>
           <t>3001085</t>
         </is>
       </c>
-      <c r="H90" s="7" t="inlineStr">
+      <c r="H90" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -4609,40 +4609,40 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B96" s="7" t="inlineStr">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C96" s="5" t="inlineStr">
         <is>
           <t>Soothing Toning Lotion
 Tónico Suave Hidratante Rosto e Olhos
 200 ml</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D96" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/soothing-toning-lotion-3001045.html</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr"/>
-      <c r="F96" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G96" s="7" t="inlineStr">
+      <c r="E96" s="5" t="inlineStr"/>
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
         <is>
           <t>3001045</t>
         </is>
       </c>
-      <c r="H96" s="7" t="inlineStr">
+      <c r="H96" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -9849,40 +9849,40 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>Sabal Argeal Shampooing Quotidien Sébo-Absorbant
 Champô Sebo-absorvente Cabeelo Oleoso
 200 ml</t>
         </is>
       </c>
-      <c r="D64" s="7" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sabal-argeal-shampooing-quotidien-sebo-absorbant-8471871.html</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr"/>
-      <c r="F64" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="E64" s="5" t="inlineStr"/>
+      <c r="F64" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
         <is>
           <t>8471871</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H64" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -10890,40 +10890,40 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Chamomile Brightening Blond Hair Spray
 Spray Camomila Aclarador 3-em-1 Cabelo Loiro
 100 ml</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/chamomile-brightening-blond-hair-spray-7615327.html</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>7615327</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -11370,40 +11370,40 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Cupuaçu Repairing CICA-shampoo
 Champô Cupuaçu Nutre Repara Cabelo Muito Seco
 200 ml</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cupuacu-repairing-cica-shampoo-8500174.html</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr"/>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>8500174</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -13100,43 +13100,43 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B70" s="7" t="inlineStr">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C70" s="7" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>Oat&amp;Ceramide Ultra-Gentle Dry Shampoo Dark
 Champô Seco Aveia Ultra-Suave Cabelo Castanho</t>
         </is>
       </c>
-      <c r="D70" s="7" t="inlineStr">
+      <c r="D70" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/oatandceramide-ultra-gentle-dry-shampoo-dark-341982.html</t>
         </is>
       </c>
-      <c r="E70" s="7" t="inlineStr">
+      <c r="E70" s="5" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F70" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="inlineStr">
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
         <is>
           <t>7831154</t>
         </is>
       </c>
-      <c r="H70" s="7" t="inlineStr">
+      <c r="H70" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -14087,40 +14087,40 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B94" s="7" t="inlineStr">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C94" s="7" t="inlineStr">
+      <c r="C94" s="3" t="inlineStr">
         <is>
           <t>Tamanu &amp; Monoi Nutri-Repair Sun Shampoo
 Champô Protetor Solar Cabelo Exposto ao Sol
 200 ml</t>
         </is>
       </c>
-      <c r="D94" s="7" t="inlineStr">
+      <c r="D94" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/tamanu-and-monoi-nutri-repair-sun-shampoo-7396246.html</t>
         </is>
       </c>
-      <c r="E94" s="7" t="inlineStr"/>
-      <c r="F94" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G94" s="7" t="inlineStr">
+      <c r="E94" s="3" t="inlineStr"/>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
         <is>
           <t>7396246</t>
         </is>
       </c>
-      <c r="H94" s="7" t="inlineStr">
+      <c r="H94" s="3" t="inlineStr">
         <is>
           <t>37%</t>
         </is>
@@ -17183,40 +17183,40 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B73" s="7" t="inlineStr">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr">
+      <c r="C73" s="3" t="inlineStr">
         <is>
           <t>Triphasic Thickening Shampoo
 Champô Queda de Cabelo e Cabelo Fino
 500 ml</t>
         </is>
       </c>
-      <c r="D73" s="7" t="inlineStr">
+      <c r="D73" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-thickening-shampoo-8602495.html</t>
         </is>
       </c>
-      <c r="E73" s="7" t="inlineStr"/>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G73" s="7" t="inlineStr">
+      <c r="E73" s="3" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
         <is>
           <t>8602495</t>
         </is>
       </c>
-      <c r="H73" s="7" t="inlineStr">
+      <c r="H73" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -17263,40 +17263,40 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B75" s="7" t="inlineStr">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C75" s="7" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr">
         <is>
           <t>Volumea Volumizing Foam
 Espuma Volumizadora Cabelo Fino sem Volume
 200 ml</t>
         </is>
       </c>
-      <c r="D75" s="7" t="inlineStr">
+      <c r="D75" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/volumea-volumizing-foam-5520281.html</t>
         </is>
       </c>
-      <c r="E75" s="7" t="inlineStr"/>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G75" s="7" t="inlineStr">
+      <c r="E75" s="3" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
         <is>
           <t>5520281</t>
         </is>
       </c>
-      <c r="H75" s="7" t="inlineStr">
+      <c r="H75" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -17941,43 +17941,43 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>7434602</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19330,40 +19330,40 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>Protect AC Mattifying Fluid SPF50+
 Protetor Solar Fluido Mate Rosto Pele Oleosa
 40ml</t>
         </is>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-ac-mattifying-fluid-spf50-5782463.html</t>
         </is>
       </c>
-      <c r="E48" s="7" t="inlineStr"/>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="E48" s="3" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
         <is>
           <t>5782463</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H48" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19528,40 +19528,40 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Protect Invisible Fluid SPF50+
 Protetor Solar Fluido Rosto Pele Oleosa
 40ml</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-invisible-fluid-spf50-6902190.html</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr"/>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>6902190</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -19608,40 +19608,40 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Protect Kids Chlidren Spray SPF50+
 Protetor Solar Spray Rosto Corpo Criança
 200ml</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-kids-chlidren-spray-spf50-5782491.html</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>5782491</t>
         </is>
       </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -24719,38 +24719,38 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>7434602</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
@@ -27642,38 +27642,38 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="7" t="inlineStr">
+      <c r="A81" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B81" s="7" t="inlineStr">
+      <c r="B81" s="3" t="inlineStr">
         <is>
           <t>Oat&amp;Ceramide Ultra-Gentle Dry Shampoo Dark
 Champô Seco Aveia Ultra-Suave Cabelo Castanho</t>
         </is>
       </c>
-      <c r="C81" s="7" t="inlineStr">
+      <c r="C81" s="3" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D81" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="inlineStr">
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
         <is>
           <t>7831154</t>
         </is>
       </c>
-      <c r="F81" s="7" t="inlineStr">
+      <c r="F81" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="G81" s="7" t="inlineStr">
+      <c r="G81" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/oatandceramide-ultra-gentle-dry-shampoo-dark-341982.html</t>
         </is>

</xml_diff>

<commit_message>
chore: run 2026-03-24 14:16 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_24_03_2026.xlsx
+++ b/logs/Consolidado_24_03_2026.xlsx
@@ -641,7 +641,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -660,7 +660,7 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -676,10 +676,10 @@
         <v>80</v>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -698,7 +698,7 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>2</v>
@@ -717,7 +717,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -13887,80 +13887,80 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C89" s="5" t="inlineStr">
+      <c r="C89" s="7" t="inlineStr">
         <is>
           <t>Shampooing Sec Séboréductreu à l'Ortie
 Champô Seco de Limpeza para Cabelo Oleoso
 150 ml</t>
         </is>
       </c>
-      <c r="D89" s="5" t="inlineStr">
+      <c r="D89" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/shampooing-sec-seboreductreu-a-lortie-3688155.html</t>
         </is>
       </c>
-      <c r="E89" s="5" t="inlineStr"/>
-      <c r="F89" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G89" s="5" t="inlineStr">
+      <c r="E89" s="7" t="inlineStr"/>
+      <c r="F89" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr">
         <is>
           <t>3688155</t>
         </is>
       </c>
-      <c r="H89" s="5" t="inlineStr">
+      <c r="H89" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C90" s="3" t="inlineStr">
+      <c r="C90" s="7" t="inlineStr">
         <is>
           <t>Sweet Almond Cold Wax Small Strips
 Bandas Depilatórias Amêndoa Cera Fria Rosto
 6 un</t>
         </is>
       </c>
-      <c r="D90" s="3" t="inlineStr">
+      <c r="D90" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/sweet-almond-cold-wax-small-strips-3689514.html</t>
         </is>
       </c>
-      <c r="E90" s="3" t="inlineStr"/>
-      <c r="F90" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G90" s="3" t="inlineStr">
+      <c r="E90" s="7" t="inlineStr"/>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G90" s="7" t="inlineStr">
         <is>
           <t>3689514</t>
         </is>
       </c>
-      <c r="H90" s="3" t="inlineStr">
+      <c r="H90" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>

</xml_diff>

<commit_message>
chore: run 2026-03-24 18:03 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_24_03_2026.xlsx
+++ b/logs/Consolidado_24_03_2026.xlsx
@@ -679,7 +679,7 @@
         <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -714,10 +714,10 @@
         <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -19608,40 +19608,40 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="inlineStr">
-        <is>
-          <t>24/03/2026</t>
-        </is>
-      </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>Protect Kids Chlidren Spray SPF50+
 Protetor Solar Spray Rosto Corpo Criança
 200ml</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D55" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/protect-kids-chlidren-spray-spf50-5782491.html</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr"/>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="E55" s="7" t="inlineStr"/>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
         <is>
           <t>5782491</t>
         </is>
       </c>
-      <c r="H55" s="5" t="inlineStr">
+      <c r="H55" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>

</xml_diff>